<commit_message>
fix: remove duplicacao do ESTAPAR entre a carga do Hyper e a base do Yuri
A carga que fiz da aba Hyper do P&L trouxe o ESTAPAR de novo, que ja estava na Base
Unificada como BR02/Multisector — mesma receita, mesmo mes, R$ 324.137 contados em dobro.
Por decisao da Amanda, mantida a linha do Yuri (classificacao de metas) e removida a minha
carga; as linhas do Yuri receberam o PEP BR02CLP00103.1.1, que e o mesmo contrato
213775_ESTAPAR na empresa BR02 da linha.
Conferidos os outros 3 clientes presentes nas duas fontes (Grupo Elfa, Odontoprev, Unimed
Nacional): projetos e valores diferentes, nao sao duplicata.
Receita realizada do Q2: 63.808.968 | 99,8% com PEP (6 linhas / R$ 120.644 sem).

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/grupo_mult_q4.xlsx
+++ b/backend/grupo_mult_q4.xlsx
@@ -442,7 +442,7 @@
     <col width="21" customWidth="1" min="10" max="10"/>
     <col width="23" customWidth="1" min="11" max="11"/>
     <col width="21" customWidth="1" min="12" max="12"/>
-    <col width="23" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1624,13 +1624,13 @@
         <v>-280905.72</v>
       </c>
       <c r="K20" s="2" t="n">
-        <v>0</v>
+        <v>-175010.41375</v>
       </c>
       <c r="L20" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M20" s="2" t="n">
-        <v>-280905.72</v>
+        <v>-455916.13375</v>
       </c>
     </row>
     <row r="21">
@@ -2214,13 +2214,13 @@
         <v>137151.65</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>-149451.3415277778</v>
+        <v>-137211.3415277778</v>
       </c>
       <c r="L30" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M30" s="2" t="n">
-        <v>-12299.69152777779</v>
+        <v>-59.691527777788</v>
       </c>
     </row>
     <row r="31">

</xml_diff>